<commit_message>
ajout des substances manquante PCB
</commit_message>
<xml_diff>
--- a/Br_E_default.xlsx
+++ b/Br_E_default.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1608,12 +1608,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>As</t>
+          <t>fraction c10-c12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1622,7 +1622,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.05459508974683887</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1631,24 +1631,24 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>Mackay_97</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>n=185, mode=strict, r²=0.31</t>
+          <t>Mackay_97 feuille : BCF sensible à conc_air — utiliser une mesure représentative du site</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>fraction c12-c16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.4518451780941289</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1666,19 +1666,19 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>Mackay_97</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>n=316, mode=strict, r²=0.09</t>
+          <t>Mackay_97 feuille : BCF sensible à conc_air — utiliser une mesure représentative du site</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>As</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.05920527651024618</v>
+        <v>0.05459508974683887</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1706,14 +1706,14 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>n=37, mode=strict, r²=0.01</t>
+          <t>n=185, mode=strict, r²=0.31</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cr</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.04026256938211789</v>
+        <v>0.4518451780941289</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1741,14 +1741,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>n=86, mode=strict, r²=0.02</t>
+          <t>n=316, mode=strict, r²=0.09</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cu</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.2224822586729524</v>
+        <v>0.05920527651024618</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1776,14 +1776,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>n=181, mode=strict, r²=0.21</t>
+          <t>n=37, mode=strict, r²=0.01</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hg</t>
+          <t>Cr</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.03629952985020955</v>
+        <v>0.04026256938211789</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1811,14 +1811,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>n=21, mode=strict, r²=0.78</t>
+          <t>n=86, mode=strict, r²=0.02</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mo</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1.240216797566293</v>
+        <v>0.2224822586729524</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1846,14 +1846,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>n=17, mode=strict, r²=0.35</t>
+          <t>n=181, mode=strict, r²=0.21</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Hg</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.1031983458305061</v>
+        <v>0.03629952985020955</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1881,14 +1881,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>n=89, mode=strict, r²=0.05</t>
+          <t>n=21, mode=strict, r²=0.78</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pb</t>
+          <t>Mo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1902,7 +1902,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.03147654206824373</v>
+        <v>1.240216797566293</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1916,14 +1916,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>n=218, mode=strict, r²=0.05</t>
+          <t>n=17, mode=strict, r²=0.35</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sb</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.01599961482226948</v>
+        <v>0.1031983458305061</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1951,14 +1951,14 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>n=46, mode=strict, r²=0.35</t>
+          <t>n=89, mode=strict, r²=0.05</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Se</t>
+          <t>Pb</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.156336100318486</v>
+        <v>0.03147654206824373</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1986,14 +1986,14 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>n=18, mode=assoupli, r²=0.84</t>
+          <t>n=218, mode=strict, r²=0.05</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tl</t>
+          <t>Sb</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.9345736398497123</v>
+        <v>0.01599961482226948</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2021,14 +2021,14 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>n=41, mode=strict, r²=0.37</t>
+          <t>n=46, mode=strict, r²=0.35</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Se</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.0297085951764288</v>
+        <v>1.156336100318486</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2056,14 +2056,14 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>n=14, mode=strict, r²=0.13</t>
+          <t>n=18, mode=assoupli, r²=0.84</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Zn</t>
+          <t>Tl</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.3856630218895464</v>
+        <v>0.9345736398497123</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2091,19 +2091,19 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>n=194, mode=strict, r²=0.20</t>
+          <t>n=41, mode=strict, r²=0.37</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PCB101</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.09129093371629268</v>
+        <v>0.0297085951764288</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2121,24 +2121,24 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>n=27, r²=0.75</t>
+          <t>n=14, mode=strict, r²=0.13</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PCB118</t>
+          <t>Zn</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2690443064740529</v>
+        <v>0.3856630218895464</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2156,19 +2156,19 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>n=16, r²=0.02</t>
+          <t>n=194, mode=strict, r²=0.20</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PCB138</t>
+          <t>PCB101</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2182,7 +2182,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.1112016124728972</v>
+        <v>0.09129093371629268</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2196,14 +2196,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>n=26, r²=0.67</t>
+          <t>n=27, r²=0.75</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PCB153</t>
+          <t>PCB118</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2217,7 +2217,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.1111503830148127</v>
+        <v>0.2690443064740529</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2226,19 +2226,19 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>n=27, r²=0.66</t>
+          <t>n=16, r²=0.02</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PCB180</t>
+          <t>PCB138</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2252,7 +2252,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1538629773937793</v>
+        <v>0.1112016124728972</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2261,19 +2261,19 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPOP_OLS (régression)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>n=16, r²=0.31</t>
+          <t>n=26, r²=0.67</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PCB28</t>
+          <t>PCB153</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2.643312101910828</v>
+        <v>0.1111503830148127</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2296,45 +2296,115 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPOP_OLS (régression)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>n=3, intervalle [1.85;2.68]</t>
+          <t>n=27, r²=0.66</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>PCB180</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>légumes_feuilles</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0.1538629773937793</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>n=16, r²=0.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PCB28</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>légumes_feuilles</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>2.643312101910828</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>n=3, intervalle [1.85;2.68]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>PCB52</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>légumes_feuilles</t>
         </is>
       </c>
-      <c r="D57" t="n">
+      <c r="D59" t="n">
         <v>2.430863254392666</v>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>mg/kg_vegsec / (mg/kg_sol)</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
         <is>
           <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>n=24, r²=0.22</t>
         </is>
@@ -2351,7 +2421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3543,12 +3613,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>As</t>
+          <t>fraction c10-c12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3557,7 +3627,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.03488401370159511</v>
+        <v>2e-06</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -3566,24 +3636,24 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>PlantX</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>n=163, mode=strict, r²=0.32</t>
+          <t>log Kow=5.31 &gt; 5.0 : PlantX non validé pour les HAP lourds — résultat à interpréter avec précaution; PlantX validé uniquement sur tomate/haricot</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>fraction c12-c16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3592,7 +3662,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.2039666097917775</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -3601,19 +3671,19 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>PlantX</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>n=129, mode=strict, r²=0.06</t>
+          <t>log Kow=6.69 &gt; 5.0 : PlantX non validé pour les HAP lourds — résultat à interpréter avec précaution; PlantX validé uniquement sur tomate/haricot</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>As</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3627,7 +3697,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.0799232590339426</v>
+        <v>0.03488401370159511</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -3641,14 +3711,14 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>n=20, mode=strict, r²=0.43</t>
+          <t>n=163, mode=strict, r²=0.32</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cr</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3662,7 +3732,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.03549158310753732</v>
+        <v>0.2039666097917775</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -3676,14 +3746,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>n=75, mode=strict, r²=0.24</t>
+          <t>n=129, mode=strict, r²=0.06</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cu</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3697,7 +3767,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1880608229486312</v>
+        <v>0.0799232590339426</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -3711,14 +3781,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>n=143, mode=strict, r²=0.32</t>
+          <t>n=20, mode=strict, r²=0.43</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hg</t>
+          <t>Cr</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3732,7 +3802,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.4957675574816767</v>
+        <v>0.03549158310753732</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -3746,14 +3816,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>n=33, mode=strict, r²=0.16</t>
+          <t>n=75, mode=strict, r²=0.24</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mo</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3767,7 +3837,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>7.01640411667543</v>
+        <v>0.1880608229486312</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -3781,14 +3851,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>n=12, mode=assoupli, r²=0.38</t>
+          <t>n=143, mode=strict, r²=0.32</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Hg</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3802,7 +3872,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.01537562223828391</v>
+        <v>0.4957675574816767</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3816,14 +3886,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>n=59, mode=strict, r²=0.09</t>
+          <t>n=33, mode=strict, r²=0.16</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pb</t>
+          <t>Mo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3837,7 +3907,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.01214235234504182</v>
+        <v>7.01640411667543</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -3851,14 +3921,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>n=126, mode=strict, r²=0.04</t>
+          <t>n=12, mode=assoupli, r²=0.38</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sb</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3872,7 +3942,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.005969576468661911</v>
+        <v>0.01537562223828391</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3886,14 +3956,14 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>n=13, mode=assoupli, r²=0.05</t>
+          <t>n=59, mode=strict, r²=0.09</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Se</t>
+          <t>Pb</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3907,7 +3977,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.899144482330935</v>
+        <v>0.01214235234504182</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -3921,14 +3991,14 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>n=20, mode=strict, r²=1.00</t>
+          <t>n=126, mode=strict, r²=0.04</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tl</t>
+          <t>Sb</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3942,7 +4012,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.5963599259594181</v>
+        <v>0.005969576468661911</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3956,14 +4026,14 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>n=2, mode=assoupli</t>
+          <t>n=13, mode=assoupli, r²=0.05</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Se</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3977,7 +4047,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.02248013774430245</v>
+        <v>1.899144482330935</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -3991,14 +4061,14 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>n=12, mode=strict, r²=0.62</t>
+          <t>n=20, mode=strict, r²=1.00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Zn</t>
+          <t>Tl</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4012,7 +4082,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.1797789670545932</v>
+        <v>0.5963599259594181</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -4026,19 +4096,19 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>n=151, mode=strict, r²=0.05</t>
+          <t>n=2, mode=assoupli</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PCB101</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -4047,7 +4117,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2.590673575129534</v>
+        <v>0.02248013774430245</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -4056,24 +4126,24 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>n=11, r²=0.23</t>
+          <t>n=12, mode=strict, r²=0.62</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PCB118</t>
+          <t>Zn</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -4082,7 +4152,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2903216575091576</v>
+        <v>0.1797789670545932</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -4091,19 +4161,19 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>n=16, r²=0.12</t>
+          <t>n=151, mode=strict, r²=0.05</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PCB138</t>
+          <t>PCB101</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4117,7 +4187,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5.310030971564776</v>
+        <v>2.590673575129534</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -4126,19 +4196,19 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>n=11, r²=0.50</t>
+          <t>n=11, r²=0.23</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PCB153</t>
+          <t>PCB118</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4152,7 +4222,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>7.803766869075332</v>
+        <v>0.2903216575091576</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -4161,19 +4231,19 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>n=11, r²=0.58</t>
+          <t>n=16, r²=0.12</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PCB180</t>
+          <t>PCB138</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4187,7 +4257,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.43122035360069</v>
+        <v>5.310030971564776</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -4196,19 +4266,19 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPOP_OLS (régression)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>n=9, r²=0.01</t>
+          <t>n=11, r²=0.50</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PCB28</t>
+          <t>PCB153</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4222,7 +4292,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.521739130434782</v>
+        <v>7.803766869075332</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -4231,45 +4301,115 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPOP_OLS (régression)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>n=3, intervalle [0.253;75.1]</t>
+          <t>n=11, r²=0.58</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>PCB180</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>légumes_fruits</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0.43122035360069</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>n=9, r²=0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PCB28</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>légumes_fruits</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1.521739130434782</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>n=3, intervalle [0.253;75.1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>PCB52</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>légumes_fruits</t>
         </is>
       </c>
-      <c r="D57" t="n">
+      <c r="D59" t="n">
         <v>1.891252955082742</v>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>mg/kg_vegsec / (mg/kg_sol)</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
         <is>
           <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>n=11, r²=0.04</t>
         </is>
@@ -4286,7 +4426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5474,12 +5614,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>As</t>
+          <t>fraction c10-c12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5488,7 +5628,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.03728288890114557</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -5497,24 +5637,24 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>PlantX</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>n=24, mode=strict, r²=0.47</t>
+          <t>log Kow=5.31 &gt; 5.0 : PlantX non validé pour les HAP lourds — résultat à interpréter avec précaution</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>fraction c12-c16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5523,7 +5663,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.3139843508546843</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -5532,19 +5672,19 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>PlantX</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>n=16, mode=strict, r²=0.30</t>
+          <t>log Kow=6.69 &gt; 5.0 : PlantX non validé pour les HAP lourds — résultat à interpréter avec précaution</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>As</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -5558,7 +5698,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.009686394262829419</v>
+        <v>0.03728288890114557</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -5572,14 +5712,14 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>n=2, mode=assoupli</t>
+          <t>n=24, mode=strict, r²=0.47</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cr</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -5593,7 +5733,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.03867943157775314</v>
+        <v>0.3139843508546843</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -5607,14 +5747,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>n=28, mode=assoupli, r²=0.20</t>
+          <t>n=16, mode=strict, r²=0.30</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cu</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -5628,7 +5768,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.1794995869389268</v>
+        <v>0.009686394262829419</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -5642,14 +5782,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>n=21, mode=strict, r²=0.80</t>
+          <t>n=2, mode=assoupli</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hg</t>
+          <t>Cr</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -5663,7 +5803,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.395265723523257</v>
+        <v>0.03867943157775314</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -5677,14 +5817,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>n=4, mode=assoupli, r²=0.37</t>
+          <t>n=28, mode=assoupli, r²=0.20</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mo</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5698,7 +5838,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.144709315008348</v>
+        <v>0.1794995869389268</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -5712,14 +5852,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>n=2, mode=assoupli</t>
+          <t>n=21, mode=strict, r²=0.80</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Hg</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5733,7 +5873,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.03887583170789653</v>
+        <v>0.395265723523257</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -5747,14 +5887,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>n=46, mode=assoupli, r²=0.08</t>
+          <t>n=4, mode=assoupli, r²=0.37</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pb</t>
+          <t>Mo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5768,7 +5908,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.009217327386540221</v>
+        <v>3.144709315008348</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -5782,14 +5922,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>n=19, mode=strict, r²=0.15</t>
+          <t>n=2, mode=assoupli</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sb</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5803,7 +5943,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.04969273429743422</v>
+        <v>0.03887583170789653</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -5817,14 +5957,14 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>n=6, mode=assoupli, r²=0.39</t>
+          <t>n=46, mode=assoupli, r²=0.08</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Zn</t>
+          <t>Pb</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5838,7 +5978,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.220306319048768</v>
+        <v>0.009217327386540221</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -5852,19 +5992,19 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>n=21, mode=strict, r²=0.69</t>
+          <t>n=19, mode=strict, r²=0.15</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PCB101</t>
+          <t>Sb</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5873,7 +6013,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.1753297554694793</v>
+        <v>0.04969273429743422</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -5882,24 +6022,24 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>n=25, r²=0.51</t>
+          <t>n=6, mode=assoupli, r²=0.39</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PCB118</t>
+          <t>Zn</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5908,7 +6048,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.6045383045490131</v>
+        <v>0.220306319048768</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -5917,19 +6057,19 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>n=22, r²=1.00</t>
+          <t>n=21, mode=strict, r²=0.69</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PCB138</t>
+          <t>PCB101</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5943,7 +6083,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.2321966020959541</v>
+        <v>0.1753297554694793</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -5957,14 +6097,14 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>n=34, r²=0.81</t>
+          <t>n=25, r²=0.51</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PCB153</t>
+          <t>PCB118</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5978,7 +6118,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.1758946319581776</v>
+        <v>0.6045383045490131</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -5992,14 +6132,14 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>n=37, r²=0.71</t>
+          <t>n=22, r²=1.00</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PCB180</t>
+          <t>PCB138</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6013,7 +6153,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.172114538504629</v>
+        <v>0.2321966020959541</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -6027,14 +6167,14 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>n=30, r²=0.69</t>
+          <t>n=34, r²=0.81</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PCB28</t>
+          <t>PCB153</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6048,7 +6188,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.71827562740666</v>
+        <v>0.1758946319581776</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -6062,40 +6202,110 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>n=10, r²=1.00</t>
+          <t>n=37, r²=0.71</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>PCB180</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>légumes_racines</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0.172114538504629</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>BAPPOP_OLS (régression)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>n=30, r²=0.69</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PCB28</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>légumes_racines</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.71827562740666</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>BAPPOP_OLS (régression)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>n=10, r²=1.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>PCB52</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>légumes_racines</t>
         </is>
       </c>
-      <c r="D54" t="n">
+      <c r="D56" t="n">
         <v>1.067809498270646</v>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>mg/kg_vegsec / (mg/kg_sol)</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
         <is>
           <t>BAPPOP_OLS (régression)</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>n=26, r²=0.95</t>
         </is>
@@ -6112,7 +6322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7300,12 +7510,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>As</t>
+          <t>fraction c10-c12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -7314,7 +7524,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.1237761720768556</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7323,24 +7533,24 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>PlantX</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>n=50, mode=strict, r²=0.72</t>
+          <t>log Kow=5.31 &gt; 5.0 : PlantX non validé pour les HAP lourds — résultat à interpréter avec précaution</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>fraction c12-c16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Métal</t>
+          <t>HCT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -7349,7 +7559,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.1391848673920042</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7358,19 +7568,19 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
+          <t>PlantX</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>n=103, mode=strict, r²=0.76</t>
+          <t>log Kow=6.69 &gt; 5.0 : PlantX non validé pour les HAP lourds — résultat à interpréter avec précaution</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>As</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7384,7 +7594,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3.361890228297017</v>
+        <v>0.1237761720768556</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7398,14 +7608,14 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>n=11, mode=assoupli, r²=0.84</t>
+          <t>n=50, mode=strict, r²=0.72</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cr</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7419,7 +7629,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.05032764974070156</v>
+        <v>0.1391848673920042</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7433,14 +7643,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>n=28, mode=assoupli, r²=0.28</t>
+          <t>n=103, mode=strict, r²=0.76</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cu</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7454,7 +7664,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.3403394091854428</v>
+        <v>3.361890228297017</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7468,14 +7678,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>n=52, mode=strict, r²=0.28</t>
+          <t>n=11, mode=assoupli, r²=0.84</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hg</t>
+          <t>Cr</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7489,7 +7699,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.9009113474307318</v>
+        <v>0.05032764974070156</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7503,14 +7713,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>n=5, mode=assoupli, r²=1.00</t>
+          <t>n=28, mode=assoupli, r²=0.28</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mo</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7524,7 +7734,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.4128488535855251</v>
+        <v>0.3403394091854428</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7538,14 +7748,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>n=9, mode=assoupli, r²=0.45</t>
+          <t>n=52, mode=strict, r²=0.28</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Hg</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7559,7 +7769,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2408144874833058</v>
+        <v>0.9009113474307318</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7573,14 +7783,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>n=29, mode=strict, r²=0.10</t>
+          <t>n=5, mode=assoupli, r²=1.00</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pb</t>
+          <t>Mo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7594,7 +7804,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.145921712564457</v>
+        <v>0.4128488535855251</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7608,14 +7818,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>n=30, mode=strict, r²=0.08</t>
+          <t>n=9, mode=assoupli, r²=0.45</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Sb</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7629,7 +7839,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.0173809673145142</v>
+        <v>0.2408144874833058</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -7643,14 +7853,14 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>n=11, mode=assoupli, r²=0.15</t>
+          <t>n=29, mode=strict, r²=0.10</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tl</t>
+          <t>Pb</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7664,7 +7874,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.145921712564457</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -7678,14 +7888,14 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>n=1, mode=assoupli</t>
+          <t>n=30, mode=strict, r²=0.08</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Zn</t>
+          <t>Sb</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7699,7 +7909,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.3437001375505004</v>
+        <v>0.0173809673145142</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -7713,19 +7923,19 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>n=58, mode=strict, r²=0.19</t>
+          <t>n=11, mode=assoupli, r²=0.15</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PCB101</t>
+          <t>Tl</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -7734,7 +7944,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.09900990099009901</v>
+        <v>0.2325581395348837</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -7743,24 +7953,24 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>n=13, r²=0.46</t>
+          <t>n=1, mode=assoupli</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PCB118</t>
+          <t>Zn</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>Métal</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -7769,7 +7979,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.03363411893844281</v>
+        <v>0.3437001375505004</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -7778,19 +7988,19 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPET_OLS (moy_geom_cs_absent)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>n=19, r²=0.66</t>
+          <t>n=58, mode=strict, r²=0.19</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PCB138</t>
+          <t>PCB101</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7804,7 +8014,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.08914075455602107</v>
+        <v>0.09900990099009901</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -7813,19 +8023,19 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>BAPPOP_OLS (régression)</t>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>n=19, r²=0.70</t>
+          <t>n=13, r²=0.46</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PCB153</t>
+          <t>PCB118</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7839,7 +8049,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.1010100232343111</v>
+        <v>0.03363411893844281</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -7853,14 +8063,14 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>n=19, r²=0.74</t>
+          <t>n=19, r²=0.66</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PCB180</t>
+          <t>PCB138</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7874,7 +8084,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.0521844245387167</v>
+        <v>0.08914075455602107</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -7888,14 +8098,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>n=13, r²=0.74</t>
+          <t>n=19, r²=0.70</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PCB28</t>
+          <t>PCB153</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -7909,7 +8119,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.3378378378378378</v>
+        <v>0.1010100232343111</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -7918,45 +8128,115 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>BAPPOP (médiane, r²≤0.5)</t>
+          <t>BAPPOP_OLS (régression)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>n=7, r²=0.16</t>
+          <t>n=19, r²=0.74</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>PCB180</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>tubercules</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.0521844245387167</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>BAPPOP_OLS (régression)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>n=13, r²=0.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>PCB28</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>tubercules</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0.3378378378378378</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>BAPPOP (médiane, r²≤0.5)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>n=7, r²=0.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>PCB52</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>PCB</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>tubercules</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D57" t="n">
         <v>0.3326680672268908</v>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>mg/kg_vegsec / (mg/kg_sol)</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>mg/kg_vegsec / (mg/kg_sol)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
         <is>
           <t>BAPPOP (médiane, r²≤0.5)</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>n=8, r²=0.08</t>
         </is>

</xml_diff>